<commit_message>
[2026-07-22] 中银消金 - 生成函数导入文件(.fun)及function_definitions
</commit_message>
<xml_diff>
--- a/日常/2026-07-22/指标规则智能配置-中银消金风险部v3_function_forge.xlsx
+++ b/日常/2026-07-22/指标规则智能配置-中银消金风险部v3_function_forge.xlsx
@@ -548,7 +548,11 @@
           <t>同盾科技</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>FHKD000001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -589,7 +593,11 @@
           <t>同盾科技</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>SHKD000002</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -630,7 +638,11 @@
           <t>同盾科技</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>SHKD000003</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -853,7 +865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">

</xml_diff>